<commit_message>
procurement: fully-loaded top-10 container, enriched from price lists
Filled KRW FOB price + carton specs for 3 SKUs from price lists/order
(Round Lab Dokdo, Celimax Toner, Celimax Retinol). For 7 SKUs without a
price list in the repo (Enough, Manyo, JMSolution, Etude), imputed KRW
from Raketa actual RUB cost and estimated per-unit weight (orange cells).
Quantities scaled so the container loads to 26.0 t (100%, 113 474 units).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XzNBEf4vaaEHRqeR8ZkfFA
</commit_message>
<xml_diff>
--- a/outputs/procurement/container_top10_2026-06-30.xlsx
+++ b/outputs/procurement/container_top10_2026-06-30.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,8 +36,12 @@
       <b val="1"/>
       <color rgb="00C00000"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00C55A11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +56,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -86,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -94,10 +103,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -463,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X17"/>
+  <dimension ref="A1:X19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -619,17 +629,19 @@
           <t>ROUND LAB 1025 DOKDO CLEANSER_150ml</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>8809738608364</v>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>8809738608364</t>
+        </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>21144</v>
+        <v>37844</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>6220</v>
       </c>
       <c r="F3" s="4">
-        <f>IF(OR($G3="",$E3=""),"",$J3*$G3*$E3)</f>
+        <f>$J3*$G3*$E3</f>
         <v/>
       </c>
       <c r="G3" s="4" t="n">
@@ -642,47 +654,47 @@
         <v>7</v>
       </c>
       <c r="J3" s="4">
-        <f>IF($G3="","",ROUNDUP($D3/$G3,0))</f>
+        <f>ROUNDUP($D3/$G3,0)</f>
         <v/>
       </c>
       <c r="K3" s="4">
-        <f>IF($J3="","",$J3*$H3)</f>
+        <f>$J3*$H3</f>
         <v/>
       </c>
       <c r="L3" s="4">
-        <f>IF($K3="","",SUMIF($A:$A,$A3,$K:$K))</f>
+        <f>SUMIF($A:$A,$A3,$K:$K)</f>
         <v/>
       </c>
       <c r="M3" s="4">
-        <f>IF($J3="","",$J3*$I3)</f>
+        <f>$J3*$I3</f>
         <v/>
       </c>
       <c r="N3" s="4">
-        <f>IF($E3="","",$E3*$X$1)</f>
+        <f>$E3*$X$1</f>
         <v/>
       </c>
       <c r="O3" s="4">
-        <f>IF($G3="","",$I3/$G3)</f>
+        <f>$I3/$G3</f>
         <v/>
       </c>
       <c r="P3" s="4">
-        <f>IF($O3="","",$O3*$X$2)</f>
+        <f>$O3*$X$2</f>
         <v/>
       </c>
       <c r="Q3" s="4">
-        <f>IF($N3="","",$N3+$P3)</f>
+        <f>$N3+$P3</f>
         <v/>
       </c>
       <c r="R3" s="4">
-        <f>IF($J3="","",$J3*$G3*$N3)</f>
+        <f>$J3*$G3*$N3</f>
         <v/>
       </c>
       <c r="S3" s="4">
-        <f>IF($J3="","",$J3*$G3*$P3)</f>
+        <f>$J3*$G3*$P3</f>
         <v/>
       </c>
       <c r="T3" s="4">
-        <f>IF($R3="","",$R3+$S3)</f>
+        <f>$R3+$S3</f>
         <v/>
       </c>
     </row>
@@ -697,17 +709,19 @@
           <t>Celimax Dual Barrier Creamy Toner</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
-        <v>8809606850475</v>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>8809606850475</t>
+        </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>32634</v>
+        <v>54981</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>8930</v>
+        <v>10930</v>
       </c>
       <c r="F4" s="4">
-        <f>IF(OR($G4="",$E4=""),"",$J4*$G4*$E4)</f>
+        <f>$J4*$G4*$E4</f>
         <v/>
       </c>
       <c r="G4" s="4" t="n">
@@ -717,50 +731,50 @@
         <v>0.0155</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>6.1</v>
+        <v>6.07</v>
       </c>
       <c r="J4" s="4">
-        <f>IF($G4="","",ROUNDUP($D4/$G4,0))</f>
+        <f>ROUNDUP($D4/$G4,0)</f>
         <v/>
       </c>
       <c r="K4" s="4">
-        <f>IF($J4="","",$J4*$H4)</f>
+        <f>$J4*$H4</f>
         <v/>
       </c>
       <c r="L4" s="4">
-        <f>IF($K4="","",SUMIF($A:$A,$A4,$K:$K))</f>
+        <f>SUMIF($A:$A,$A4,$K:$K)</f>
         <v/>
       </c>
       <c r="M4" s="4">
-        <f>IF($J4="","",$J4*$I4)</f>
+        <f>$J4*$I4</f>
         <v/>
       </c>
       <c r="N4" s="4">
-        <f>IF($E4="","",$E4*$X$1)</f>
+        <f>$E4*$X$1</f>
         <v/>
       </c>
       <c r="O4" s="4">
-        <f>IF($G4="","",$I4/$G4)</f>
+        <f>$I4/$G4</f>
         <v/>
       </c>
       <c r="P4" s="4">
-        <f>IF($O4="","",$O4*$X$2)</f>
+        <f>$O4*$X$2</f>
         <v/>
       </c>
       <c r="Q4" s="4">
-        <f>IF($N4="","",$N4+$P4)</f>
+        <f>$N4+$P4</f>
         <v/>
       </c>
       <c r="R4" s="4">
-        <f>IF($J4="","",$J4*$G4*$N4)</f>
+        <f>$J4*$G4*$N4</f>
         <v/>
       </c>
       <c r="S4" s="4">
-        <f>IF($J4="","",$J4*$G4*$P4)</f>
+        <f>$J4*$G4*$P4</f>
         <v/>
       </c>
       <c r="T4" s="4">
-        <f>IF($R4="","",$R4+$S4)</f>
+        <f>$R4+$S4</f>
         <v/>
       </c>
     </row>
@@ -777,62 +791,70 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>551465879</t>
+          <t>8809700320805</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
         <v>3666</v>
       </c>
-      <c r="E5" s="5" t="n"/>
+      <c r="E5" s="4" t="n">
+        <v>10130</v>
+      </c>
       <c r="F5" s="4">
-        <f>IF(OR($G5="",$E5=""),"",$J5*$G5*$E5)</f>
-        <v/>
-      </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
+        <f>$J5*$G5*$E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>5.8</v>
+      </c>
       <c r="J5" s="4">
-        <f>IF($G5="","",ROUNDUP($D5/$G5,0))</f>
+        <f>ROUNDUP($D5/$G5,0)</f>
         <v/>
       </c>
       <c r="K5" s="4">
-        <f>IF($J5="","",$J5*$H5)</f>
+        <f>$J5*$H5</f>
         <v/>
       </c>
       <c r="L5" s="4">
-        <f>IF($K5="","",SUMIF($A:$A,$A5,$K:$K))</f>
+        <f>SUMIF($A:$A,$A5,$K:$K)</f>
         <v/>
       </c>
       <c r="M5" s="4">
-        <f>IF($J5="","",$J5*$I5)</f>
+        <f>$J5*$I5</f>
         <v/>
       </c>
       <c r="N5" s="4">
-        <f>IF($E5="","",$E5*$X$1)</f>
+        <f>$E5*$X$1</f>
         <v/>
       </c>
       <c r="O5" s="4">
-        <f>IF($G5="","",$I5/$G5)</f>
+        <f>$I5/$G5</f>
         <v/>
       </c>
       <c r="P5" s="4">
-        <f>IF($O5="","",$O5*$X$2)</f>
+        <f>$O5*$X$2</f>
         <v/>
       </c>
       <c r="Q5" s="4">
-        <f>IF($N5="","",$N5+$P5)</f>
+        <f>$N5+$P5</f>
         <v/>
       </c>
       <c r="R5" s="4">
-        <f>IF($J5="","",$J5*$G5*$N5)</f>
+        <f>$J5*$G5*$N5</f>
         <v/>
       </c>
       <c r="S5" s="4">
-        <f>IF($J5="","",$J5*$G5*$P5)</f>
+        <f>$J5*$G5*$P5</f>
         <v/>
       </c>
       <c r="T5" s="4">
-        <f>IF($R5="","",$R5+$S5)</f>
+        <f>$R5+$S5</f>
         <v/>
       </c>
     </row>
@@ -847,71 +869,75 @@
           <t>ENOUGH - Collagen Moisture Essential Cream [50ml] N</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>238415286</t>
-        </is>
-      </c>
+      <c r="C6" s="4" t="inlineStr"/>
       <c r="D6" s="4" t="n">
         <v>7257</v>
       </c>
-      <c r="E6" s="5" t="n"/>
+      <c r="E6" s="5" t="n">
+        <v>2672</v>
+      </c>
       <c r="F6" s="4">
-        <f>IF(OR($G6="",$E6=""),"",$J6*$G6*$E6)</f>
-        <v/>
-      </c>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
+        <f>$J6*$G6*$E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>7.2</v>
+      </c>
       <c r="J6" s="4">
-        <f>IF($G6="","",ROUNDUP($D6/$G6,0))</f>
+        <f>ROUNDUP($D6/$G6,0)</f>
         <v/>
       </c>
       <c r="K6" s="4">
-        <f>IF($J6="","",$J6*$H6)</f>
+        <f>$J6*$H6</f>
         <v/>
       </c>
       <c r="L6" s="4">
-        <f>IF($K6="","",SUMIF($A:$A,$A6,$K:$K))</f>
+        <f>SUMIF($A:$A,$A6,$K:$K)</f>
         <v/>
       </c>
       <c r="M6" s="4">
-        <f>IF($J6="","",$J6*$I6)</f>
+        <f>$J6*$I6</f>
         <v/>
       </c>
       <c r="N6" s="4">
-        <f>IF($E6="","",$E6*$X$1)</f>
+        <f>$E6*$X$1</f>
         <v/>
       </c>
       <c r="O6" s="4">
-        <f>IF($G6="","",$I6/$G6)</f>
+        <f>$I6/$G6</f>
         <v/>
       </c>
       <c r="P6" s="4">
-        <f>IF($O6="","",$O6*$X$2)</f>
+        <f>$O6*$X$2</f>
         <v/>
       </c>
       <c r="Q6" s="4">
-        <f>IF($N6="","",$N6+$P6)</f>
+        <f>$N6+$P6</f>
         <v/>
       </c>
       <c r="R6" s="4">
-        <f>IF($J6="","",$J6*$G6*$N6)</f>
+        <f>$J6*$G6*$N6</f>
         <v/>
       </c>
       <c r="S6" s="4">
-        <f>IF($J6="","",$J6*$G6*$P6)</f>
+        <f>$J6*$G6*$P6</f>
         <v/>
       </c>
       <c r="T6" s="4">
-        <f>IF($R6="","",$R6+$S6)</f>
+        <f>$R6+$S6</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>MANYO_GALAC_VITA_SERUM</t>
+          <t>Manyo</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -919,71 +945,75 @@
           <t>Manyo_Galac_Vita_Serum</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>198156472</t>
-        </is>
-      </c>
+      <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="n">
         <v>1428</v>
       </c>
-      <c r="E7" s="5" t="n"/>
+      <c r="E7" s="5" t="n">
+        <v>11669</v>
+      </c>
       <c r="F7" s="4">
-        <f>IF(OR($G7="",$E7=""),"",$J7*$G7*$E7)</f>
-        <v/>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
+        <f>$J7*$G7*$E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>10.4</v>
+      </c>
       <c r="J7" s="4">
-        <f>IF($G7="","",ROUNDUP($D7/$G7,0))</f>
+        <f>ROUNDUP($D7/$G7,0)</f>
         <v/>
       </c>
       <c r="K7" s="4">
-        <f>IF($J7="","",$J7*$H7)</f>
+        <f>$J7*$H7</f>
         <v/>
       </c>
       <c r="L7" s="4">
-        <f>IF($K7="","",SUMIF($A:$A,$A7,$K:$K))</f>
+        <f>SUMIF($A:$A,$A7,$K:$K)</f>
         <v/>
       </c>
       <c r="M7" s="4">
-        <f>IF($J7="","",$J7*$I7)</f>
+        <f>$J7*$I7</f>
         <v/>
       </c>
       <c r="N7" s="4">
-        <f>IF($E7="","",$E7*$X$1)</f>
+        <f>$E7*$X$1</f>
         <v/>
       </c>
       <c r="O7" s="4">
-        <f>IF($G7="","",$I7/$G7)</f>
+        <f>$I7/$G7</f>
         <v/>
       </c>
       <c r="P7" s="4">
-        <f>IF($O7="","",$O7*$X$2)</f>
+        <f>$O7*$X$2</f>
         <v/>
       </c>
       <c r="Q7" s="4">
-        <f>IF($N7="","",$N7+$P7)</f>
+        <f>$N7+$P7</f>
         <v/>
       </c>
       <c r="R7" s="4">
-        <f>IF($J7="","",$J7*$G7*$N7)</f>
+        <f>$J7*$G7*$N7</f>
         <v/>
       </c>
       <c r="S7" s="4">
-        <f>IF($J7="","",$J7*$G7*$P7)</f>
+        <f>$J7*$G7*$P7</f>
         <v/>
       </c>
       <c r="T7" s="4">
-        <f>IF($R7="","",$R7+$S7)</f>
+        <f>$R7+$S7</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>MANYO_COMPLEX_AMPOULE</t>
+          <t>Manyo</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -991,71 +1021,75 @@
           <t>Manyo_Complex_Ampoule</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>198147185</t>
-        </is>
-      </c>
+      <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="n">
         <v>879</v>
       </c>
-      <c r="E8" s="5" t="n"/>
+      <c r="E8" s="5" t="n">
+        <v>16371</v>
+      </c>
       <c r="F8" s="4">
-        <f>IF(OR($G8="",$E8=""),"",$J8*$G8*$E8)</f>
-        <v/>
-      </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
+        <f>$J8*$G8*$E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>10.4</v>
+      </c>
       <c r="J8" s="4">
-        <f>IF($G8="","",ROUNDUP($D8/$G8,0))</f>
+        <f>ROUNDUP($D8/$G8,0)</f>
         <v/>
       </c>
       <c r="K8" s="4">
-        <f>IF($J8="","",$J8*$H8)</f>
+        <f>$J8*$H8</f>
         <v/>
       </c>
       <c r="L8" s="4">
-        <f>IF($K8="","",SUMIF($A:$A,$A8,$K:$K))</f>
+        <f>SUMIF($A:$A,$A8,$K:$K)</f>
         <v/>
       </c>
       <c r="M8" s="4">
-        <f>IF($J8="","",$J8*$I8)</f>
+        <f>$J8*$I8</f>
         <v/>
       </c>
       <c r="N8" s="4">
-        <f>IF($E8="","",$E8*$X$1)</f>
+        <f>$E8*$X$1</f>
         <v/>
       </c>
       <c r="O8" s="4">
-        <f>IF($G8="","",$I8/$G8)</f>
+        <f>$I8/$G8</f>
         <v/>
       </c>
       <c r="P8" s="4">
-        <f>IF($O8="","",$O8*$X$2)</f>
+        <f>$O8*$X$2</f>
         <v/>
       </c>
       <c r="Q8" s="4">
-        <f>IF($N8="","",$N8+$P8)</f>
+        <f>$N8+$P8</f>
         <v/>
       </c>
       <c r="R8" s="4">
-        <f>IF($J8="","",$J8*$G8*$N8)</f>
+        <f>$J8*$G8*$N8</f>
         <v/>
       </c>
       <c r="S8" s="4">
-        <f>IF($J8="","",$J8*$G8*$P8)</f>
+        <f>$J8*$G8*$P8</f>
         <v/>
       </c>
       <c r="T8" s="4">
-        <f>IF($R8="","",$R8+$S8)</f>
+        <f>$R8+$S8</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>MANYO</t>
+          <t>Manyo</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1063,64 +1097,68 @@
           <t>MANYO BIFIDA INFUSION SHOT AMPOULE 1DX [50ml]</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>868700077</t>
-        </is>
-      </c>
+      <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="n">
         <v>221</v>
       </c>
-      <c r="E9" s="5" t="n"/>
+      <c r="E9" s="5" t="n">
+        <v>18173</v>
+      </c>
       <c r="F9" s="4">
-        <f>IF(OR($G9="",$E9=""),"",$J9*$G9*$E9)</f>
-        <v/>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
+        <f>$J9*$G9*$E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>0.022</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>10.4</v>
+      </c>
       <c r="J9" s="4">
-        <f>IF($G9="","",ROUNDUP($D9/$G9,0))</f>
+        <f>ROUNDUP($D9/$G9,0)</f>
         <v/>
       </c>
       <c r="K9" s="4">
-        <f>IF($J9="","",$J9*$H9)</f>
+        <f>$J9*$H9</f>
         <v/>
       </c>
       <c r="L9" s="4">
-        <f>IF($K9="","",SUMIF($A:$A,$A9,$K:$K))</f>
+        <f>SUMIF($A:$A,$A9,$K:$K)</f>
         <v/>
       </c>
       <c r="M9" s="4">
-        <f>IF($J9="","",$J9*$I9)</f>
+        <f>$J9*$I9</f>
         <v/>
       </c>
       <c r="N9" s="4">
-        <f>IF($E9="","",$E9*$X$1)</f>
+        <f>$E9*$X$1</f>
         <v/>
       </c>
       <c r="O9" s="4">
-        <f>IF($G9="","",$I9/$G9)</f>
+        <f>$I9/$G9</f>
         <v/>
       </c>
       <c r="P9" s="4">
-        <f>IF($O9="","",$O9*$X$2)</f>
+        <f>$O9*$X$2</f>
         <v/>
       </c>
       <c r="Q9" s="4">
-        <f>IF($N9="","",$N9+$P9)</f>
+        <f>$N9+$P9</f>
         <v/>
       </c>
       <c r="R9" s="4">
-        <f>IF($J9="","",$J9*$G9*$N9)</f>
+        <f>$J9*$G9*$N9</f>
         <v/>
       </c>
       <c r="S9" s="4">
-        <f>IF($J9="","",$J9*$G9*$P9)</f>
+        <f>$J9*$G9*$P9</f>
         <v/>
       </c>
       <c r="T9" s="4">
-        <f>IF($R9="","",$R9+$S9)</f>
+        <f>$R9+$S9</f>
         <v/>
       </c>
     </row>
@@ -1135,64 +1173,68 @@
           <t>JMSOLUTION - Mask Pack Disney</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>214964091</t>
-        </is>
-      </c>
+      <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="4" t="n">
         <v>1224</v>
       </c>
-      <c r="E10" s="5" t="n"/>
+      <c r="E10" s="5" t="n">
+        <v>7793</v>
+      </c>
       <c r="F10" s="4">
-        <f>IF(OR($G10="",$E10=""),"",$J10*$G10*$E10)</f>
-        <v/>
-      </c>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
+        <f>$J10*$G10*$E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>12</v>
+      </c>
       <c r="J10" s="4">
-        <f>IF($G10="","",ROUNDUP($D10/$G10,0))</f>
+        <f>ROUNDUP($D10/$G10,0)</f>
         <v/>
       </c>
       <c r="K10" s="4">
-        <f>IF($J10="","",$J10*$H10)</f>
+        <f>$J10*$H10</f>
         <v/>
       </c>
       <c r="L10" s="4">
-        <f>IF($K10="","",SUMIF($A:$A,$A10,$K:$K))</f>
+        <f>SUMIF($A:$A,$A10,$K:$K)</f>
         <v/>
       </c>
       <c r="M10" s="4">
-        <f>IF($J10="","",$J10*$I10)</f>
+        <f>$J10*$I10</f>
         <v/>
       </c>
       <c r="N10" s="4">
-        <f>IF($E10="","",$E10*$X$1)</f>
+        <f>$E10*$X$1</f>
         <v/>
       </c>
       <c r="O10" s="4">
-        <f>IF($G10="","",$I10/$G10)</f>
+        <f>$I10/$G10</f>
         <v/>
       </c>
       <c r="P10" s="4">
-        <f>IF($O10="","",$O10*$X$2)</f>
+        <f>$O10*$X$2</f>
         <v/>
       </c>
       <c r="Q10" s="4">
-        <f>IF($N10="","",$N10+$P10)</f>
+        <f>$N10+$P10</f>
         <v/>
       </c>
       <c r="R10" s="4">
-        <f>IF($J10="","",$J10*$G10*$N10)</f>
+        <f>$J10*$G10*$N10</f>
         <v/>
       </c>
       <c r="S10" s="4">
-        <f>IF($J10="","",$J10*$G10*$P10)</f>
+        <f>$J10*$G10*$P10</f>
         <v/>
       </c>
       <c r="T10" s="4">
-        <f>IF($R10="","",$R10+$S10)</f>
+        <f>$R10+$S10</f>
         <v/>
       </c>
     </row>
@@ -1207,64 +1249,68 @@
           <t>Etude Baking Powder Crunch Pore Scrub</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>151313163</t>
-        </is>
-      </c>
+      <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="n">
         <v>4840</v>
       </c>
-      <c r="E11" s="5" t="n"/>
+      <c r="E11" s="5" t="n">
+        <v>6030</v>
+      </c>
       <c r="F11" s="4">
-        <f>IF(OR($G11="",$E11=""),"",$J11*$G11*$E11)</f>
-        <v/>
-      </c>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
+        <f>$J11*$G11*$E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>12.5</v>
+      </c>
       <c r="J11" s="4">
-        <f>IF($G11="","",ROUNDUP($D11/$G11,0))</f>
+        <f>ROUNDUP($D11/$G11,0)</f>
         <v/>
       </c>
       <c r="K11" s="4">
-        <f>IF($J11="","",$J11*$H11)</f>
+        <f>$J11*$H11</f>
         <v/>
       </c>
       <c r="L11" s="4">
-        <f>IF($K11="","",SUMIF($A:$A,$A11,$K:$K))</f>
+        <f>SUMIF($A:$A,$A11,$K:$K)</f>
         <v/>
       </c>
       <c r="M11" s="4">
-        <f>IF($J11="","",$J11*$I11)</f>
+        <f>$J11*$I11</f>
         <v/>
       </c>
       <c r="N11" s="4">
-        <f>IF($E11="","",$E11*$X$1)</f>
+        <f>$E11*$X$1</f>
         <v/>
       </c>
       <c r="O11" s="4">
-        <f>IF($G11="","",$I11/$G11)</f>
+        <f>$I11/$G11</f>
         <v/>
       </c>
       <c r="P11" s="4">
-        <f>IF($O11="","",$O11*$X$2)</f>
+        <f>$O11*$X$2</f>
         <v/>
       </c>
       <c r="Q11" s="4">
-        <f>IF($N11="","",$N11+$P11)</f>
+        <f>$N11+$P11</f>
         <v/>
       </c>
       <c r="R11" s="4">
-        <f>IF($J11="","",$J11*$G11*$N11)</f>
+        <f>$J11*$G11*$N11</f>
         <v/>
       </c>
       <c r="S11" s="4">
-        <f>IF($J11="","",$J11*$G11*$P11)</f>
+        <f>$J11*$G11*$P11</f>
         <v/>
       </c>
       <c r="T11" s="4">
-        <f>IF($R11="","",$R11+$S11)</f>
+        <f>$R11+$S11</f>
         <v/>
       </c>
     </row>
@@ -1279,64 +1325,68 @@
           <t>Enough 8 Peptide Full Cover Perfect Foundation 21 тон</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>170198337</t>
-        </is>
-      </c>
+      <c r="C12" s="4" t="inlineStr"/>
       <c r="D12" s="4" t="n">
         <v>991</v>
       </c>
-      <c r="E12" s="5" t="n"/>
+      <c r="E12" s="5" t="n">
+        <v>5393</v>
+      </c>
       <c r="F12" s="4">
-        <f>IF(OR($G12="",$E12=""),"",$J12*$G12*$E12)</f>
-        <v/>
-      </c>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
+        <f>$J12*$G12*$E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>0.024</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>10</v>
+      </c>
       <c r="J12" s="4">
-        <f>IF($G12="","",ROUNDUP($D12/$G12,0))</f>
+        <f>ROUNDUP($D12/$G12,0)</f>
         <v/>
       </c>
       <c r="K12" s="4">
-        <f>IF($J12="","",$J12*$H12)</f>
+        <f>$J12*$H12</f>
         <v/>
       </c>
       <c r="L12" s="4">
-        <f>IF($K12="","",SUMIF($A:$A,$A12,$K:$K))</f>
+        <f>SUMIF($A:$A,$A12,$K:$K)</f>
         <v/>
       </c>
       <c r="M12" s="4">
-        <f>IF($J12="","",$J12*$I12)</f>
+        <f>$J12*$I12</f>
         <v/>
       </c>
       <c r="N12" s="4">
-        <f>IF($E12="","",$E12*$X$1)</f>
+        <f>$E12*$X$1</f>
         <v/>
       </c>
       <c r="O12" s="4">
-        <f>IF($G12="","",$I12/$G12)</f>
+        <f>$I12/$G12</f>
         <v/>
       </c>
       <c r="P12" s="4">
-        <f>IF($O12="","",$O12*$X$2)</f>
+        <f>$O12*$X$2</f>
         <v/>
       </c>
       <c r="Q12" s="4">
-        <f>IF($N12="","",$N12+$P12)</f>
+        <f>$N12+$P12</f>
         <v/>
       </c>
       <c r="R12" s="4">
-        <f>IF($J12="","",$J12*$G12*$N12)</f>
+        <f>$J12*$G12*$N12</f>
         <v/>
       </c>
       <c r="S12" s="4">
-        <f>IF($J12="","",$J12*$G12*$P12)</f>
+        <f>$J12*$G12*$P12</f>
         <v/>
       </c>
       <c r="T12" s="4">
-        <f>IF($R12="","",$R12+$S12)</f>
+        <f>$R12+$S12</f>
         <v/>
       </c>
     </row>
@@ -1349,7 +1399,7 @@
       </c>
       <c r="C13" s="6" t="n"/>
       <c r="D13" s="7">
-        <f>SUM(D3:D12)</f>
+        <f>SUMPRODUCT(J3:J12,G3:G12)</f>
         <v/>
       </c>
       <c r="E13" s="6" t="n"/>
@@ -1357,7 +1407,10 @@
       <c r="G13" s="6" t="n"/>
       <c r="H13" s="6" t="n"/>
       <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="n"/>
+      <c r="J13" s="7">
+        <f>SUM(J3:J12)</f>
+        <v/>
+      </c>
       <c r="K13" s="7">
         <f>SUM(K3:K12)</f>
         <v/>
@@ -1413,6 +1466,13 @@
         <v/>
       </c>
     </row>
+    <row r="19">
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Оранжевые ячейки = оценка (нет прайса в файлах), уточнить у поставщика</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>